<commit_message>
SOCO: Improv: Change default settings
Jio gave list of updated default values.
</commit_message>
<xml_diff>
--- a/Document/CustomerFacing/SOCOModbusTable.xlsx
+++ b/Document/CustomerFacing/SOCOModbusTable.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Modbus Table" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3083" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3089" uniqueCount="509">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1046,6 +1046,24 @@
   </si>
   <si>
     <t xml:space="preserve">6001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voltage at or above which the mains-undervoltage condition clears. Recommended to set above Mains UV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voltage at or below which the mains-overvoltage condition clears. Recommended to set below Mains OV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mains must stay unhealthy for this duration before the unhealthy state is latched.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mains must stay healthy for this duration before the healthy state is latched.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voltage at or above which the solar-undervoltage condition clears. Recommended to set above Solar UV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voltage at or below which the solar-overvoltage condition clears. Recommended to set below Solar OV.</t>
   </si>
   <si>
     <t xml:space="preserve">0: No Action, 1:Signals start of Firmware Uploading, 2: Signals end of Firmware Uploading</t>
@@ -1455,27 +1473,15 @@
     <t xml:space="preserve">MUVR</t>
   </si>
   <si>
-    <t xml:space="preserve">Voltage at or above which the mains-undervoltage condition clears. Recommended to set above Mains UV.</t>
-  </si>
-  <si>
     <t xml:space="preserve">MOVR</t>
   </si>
   <si>
-    <t xml:space="preserve">Voltage at or below which the mains-overvoltage condition clears. Recommended to set below Mains OV.</t>
-  </si>
-  <si>
     <t xml:space="preserve">M FL</t>
   </si>
   <si>
-    <t xml:space="preserve">Mains must stay unhealthy for this duration before the unhealthy state is latched.</t>
-  </si>
-  <si>
     <t xml:space="preserve">M RT</t>
   </si>
   <si>
-    <t xml:space="preserve">Mains must stay healthy for this duration before the healthy state is latched.</t>
-  </si>
-  <si>
     <t xml:space="preserve">S UV</t>
   </si>
   <si>
@@ -1485,13 +1491,7 @@
     <t xml:space="preserve">SUVR</t>
   </si>
   <si>
-    <t xml:space="preserve">Voltage at or above which the solar-undervoltage condition clears. Recommended to set above Solar UV.</t>
-  </si>
-  <si>
     <t xml:space="preserve">SOVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voltage at or below which the solar-overvoltage condition clears. Recommended to set below Solar OV.</t>
   </si>
   <si>
     <t xml:space="preserve">S FL</t>
@@ -1699,7 +1699,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1766,15 +1766,6 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin">
-        <color rgb="FF000001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1801,7 +1792,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1844,14 +1835,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2127,7 +2110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -7370,7 +7353,7 @@
       </c>
       <c r="I193" s="7"/>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="30.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="9" t="s">
         <v>201</v>
       </c>
@@ -7395,9 +7378,11 @@
       <c r="H194" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I194" s="7"/>
-    </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I194" s="7" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="9" t="s">
         <v>203</v>
       </c>
@@ -7422,9 +7407,11 @@
       <c r="H195" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I195" s="7"/>
-    </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I195" s="7" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="9" t="s">
         <v>205</v>
       </c>
@@ -7449,9 +7436,11 @@
       <c r="H196" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I196" s="7"/>
-    </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I196" s="7" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="9" t="s">
         <v>207</v>
       </c>
@@ -7476,7 +7465,9 @@
       <c r="H197" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I197" s="7"/>
+      <c r="I197" s="7" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="9" t="s">
@@ -7532,7 +7523,7 @@
       </c>
       <c r="I199" s="7"/>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="34.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="9" t="s">
         <v>213</v>
       </c>
@@ -7557,9 +7548,11 @@
       <c r="H200" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I200" s="7"/>
-    </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I200" s="7" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="9" t="s">
         <v>215</v>
       </c>
@@ -7584,7 +7577,9 @@
       <c r="H201" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I201" s="7"/>
+      <c r="I201" s="7" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="9" t="s">
@@ -7886,12 +7881,12 @@
         <v>2</v>
       </c>
       <c r="I212" s="7" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="7" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B213" s="7" t="s">
         <v>75</v>
@@ -7909,18 +7904,18 @@
         <v>26</v>
       </c>
       <c r="G213" s="10" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="H213" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I213" s="7" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="7" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B214" s="7" t="s">
         <v>75</v>
@@ -7938,13 +7933,13 @@
         <v>26</v>
       </c>
       <c r="G214" s="10" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="H214" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I214" s="7" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="1048534" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8017,7 +8012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -10880,32 +10875,32 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="13" t="s">
-        <v>348</v>
-      </c>
-      <c r="B109" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C109" s="14" t="s">
+      <c r="A109" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="B109" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C109" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D109" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E109" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F109" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G109" s="15" t="s">
-        <v>349</v>
-      </c>
-      <c r="H109" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I109" s="14" t="s">
-        <v>350</v>
+      <c r="D109" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E109" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G109" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="H109" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I109" s="12" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10990,235 +10985,235 @@
       <c r="I112" s="7"/>
     </row>
     <row r="113" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="13" t="s">
-        <v>351</v>
-      </c>
-      <c r="B113" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C113" s="14" t="s">
+      <c r="A113" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="B113" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C113" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D113" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E113" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F113" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G113" s="15" t="s">
-        <v>352</v>
-      </c>
-      <c r="H113" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I113" s="14" t="s">
-        <v>353</v>
+      <c r="D113" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E113" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G113" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="H113" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I113" s="12" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="13" t="s">
-        <v>354</v>
-      </c>
-      <c r="B114" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C114" s="14" t="s">
+      <c r="A114" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="B114" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C114" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D114" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E114" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F114" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G114" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="H114" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I114" s="14" t="s">
-        <v>356</v>
+      <c r="D114" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E114" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G114" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="H114" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I114" s="12" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="13" t="s">
-        <v>357</v>
-      </c>
-      <c r="B115" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C115" s="14" t="s">
+      <c r="A115" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="B115" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C115" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D115" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E115" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F115" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G115" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H115" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I115" s="14" t="s">
-        <v>359</v>
+      <c r="D115" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E115" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G115" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="H115" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I115" s="12" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="B116" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C116" s="14" t="s">
+      <c r="A116" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B116" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C116" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D116" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E116" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F116" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G116" s="15" t="s">
-        <v>361</v>
-      </c>
-      <c r="H116" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I116" s="14" t="s">
-        <v>362</v>
+      <c r="D116" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E116" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G116" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="H116" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I116" s="12" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="13" t="s">
-        <v>363</v>
-      </c>
-      <c r="B117" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="C117" s="14" t="s">
+      <c r="A117" s="11" t="s">
+        <v>369</v>
+      </c>
+      <c r="B117" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="C117" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D117" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E117" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F117" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G117" s="15" t="s">
-        <v>365</v>
-      </c>
-      <c r="H117" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I117" s="14" t="s">
-        <v>366</v>
+      <c r="D117" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E117" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G117" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="H117" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I117" s="12" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="13" t="s">
-        <v>367</v>
-      </c>
-      <c r="B118" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="C118" s="14" t="s">
+      <c r="A118" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="B118" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="C118" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D118" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E118" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F118" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G118" s="15" t="s">
-        <v>368</v>
-      </c>
-      <c r="H118" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I118" s="14" t="s">
-        <v>369</v>
+      <c r="D118" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E118" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G118" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="H118" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I118" s="12" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="13" t="s">
+      <c r="A119" s="11" t="s">
+        <v>376</v>
+      </c>
+      <c r="B119" s="12" t="s">
         <v>370</v>
       </c>
-      <c r="B119" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="C119" s="14" t="s">
+      <c r="C119" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D119" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E119" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F119" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G119" s="15" t="s">
-        <v>371</v>
-      </c>
-      <c r="H119" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I119" s="14" t="s">
-        <v>372</v>
+      <c r="D119" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E119" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G119" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="H119" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I119" s="12" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="13" t="s">
-        <v>373</v>
-      </c>
-      <c r="B120" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="C120" s="14" t="s">
+      <c r="A120" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="B120" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="C120" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D120" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E120" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F120" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G120" s="15" t="s">
-        <v>374</v>
-      </c>
-      <c r="H120" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I120" s="14" t="s">
-        <v>375</v>
+      <c r="D120" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E120" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G120" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="H120" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I120" s="12" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13398,7 +13393,7 @@
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="5" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="B198" s="5"/>
       <c r="C198" s="5"/>
@@ -13410,670 +13405,670 @@
       <c r="I198" s="5"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A199" s="14" t="s">
-        <v>377</v>
-      </c>
-      <c r="B199" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C199" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D199" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E199" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F199" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G199" s="14" t="n">
+      <c r="A199" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="B199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C199" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F199" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G199" s="12" t="n">
         <v>20001</v>
       </c>
-      <c r="H199" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I199" s="14" t="s">
-        <v>379</v>
+      <c r="H199" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I199" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A200" s="14" t="s">
-        <v>380</v>
-      </c>
-      <c r="B200" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C200" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D200" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E200" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F200" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G200" s="14" t="n">
+      <c r="A200" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="B200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C200" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F200" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G200" s="12" t="n">
         <v>20002</v>
       </c>
-      <c r="H200" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I200" s="14" t="s">
-        <v>379</v>
+      <c r="H200" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I200" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A201" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="B201" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C201" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D201" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E201" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F201" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G201" s="14" t="n">
+      <c r="A201" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="B201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C201" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F201" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G201" s="12" t="n">
         <v>20003</v>
       </c>
-      <c r="H201" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I201" s="14" t="s">
-        <v>379</v>
+      <c r="H201" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I201" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A202" s="14" t="s">
-        <v>382</v>
-      </c>
-      <c r="B202" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C202" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D202" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E202" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F202" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G202" s="14" t="n">
+      <c r="A202" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="B202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C202" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F202" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G202" s="12" t="n">
         <v>20004</v>
       </c>
-      <c r="H202" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I202" s="14" t="s">
-        <v>379</v>
+      <c r="H202" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I202" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A203" s="14" t="s">
-        <v>383</v>
-      </c>
-      <c r="B203" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C203" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D203" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E203" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F203" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G203" s="14" t="n">
+      <c r="A203" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C203" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F203" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G203" s="12" t="n">
         <v>20005</v>
       </c>
-      <c r="H203" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I203" s="14" t="s">
-        <v>379</v>
+      <c r="H203" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I203" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A204" s="14" t="s">
+      <c r="A204" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="B204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C204" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F204" s="12" t="s">
         <v>384</v>
       </c>
-      <c r="B204" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C204" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D204" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E204" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F204" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G204" s="14" t="n">
+      <c r="G204" s="12" t="n">
         <v>20006</v>
       </c>
-      <c r="H204" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I204" s="14" t="s">
-        <v>379</v>
+      <c r="H204" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I204" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A205" s="14" t="s">
+      <c r="A205" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="B205" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C205" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D205" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E205" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F205" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G205" s="12" t="n">
+        <v>20007</v>
+      </c>
+      <c r="H205" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I205" s="12" t="s">
         <v>385</v>
       </c>
-      <c r="B205" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C205" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D205" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E205" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F205" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G205" s="14" t="n">
-        <v>20007</v>
-      </c>
-      <c r="H205" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I205" s="14" t="s">
-        <v>379</v>
-      </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A206" s="14" t="s">
-        <v>386</v>
-      </c>
-      <c r="B206" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C206" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D206" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E206" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F206" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G206" s="14" t="n">
+      <c r="A206" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="B206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C206" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F206" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G206" s="12" t="n">
         <v>20008</v>
       </c>
-      <c r="H206" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I206" s="14" t="s">
-        <v>379</v>
+      <c r="H206" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I206" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A207" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="B207" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C207" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D207" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E207" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F207" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G207" s="14" t="n">
+      <c r="A207" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C207" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F207" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G207" s="12" t="n">
         <v>30001</v>
       </c>
-      <c r="H207" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I207" s="14" t="s">
-        <v>379</v>
+      <c r="H207" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I207" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A208" s="14" t="s">
-        <v>388</v>
-      </c>
-      <c r="B208" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C208" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D208" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E208" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F208" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G208" s="14" t="n">
+      <c r="A208" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="B208" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C208" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D208" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E208" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F208" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G208" s="12" t="n">
         <v>30002</v>
       </c>
-      <c r="H208" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I208" s="14" t="s">
-        <v>379</v>
+      <c r="H208" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I208" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A209" s="14" t="s">
-        <v>389</v>
-      </c>
-      <c r="B209" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C209" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D209" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E209" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F209" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G209" s="14" t="n">
+      <c r="A209" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="B209" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C209" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D209" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E209" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F209" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G209" s="12" t="n">
         <v>30003</v>
       </c>
-      <c r="H209" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I209" s="14" t="s">
-        <v>379</v>
+      <c r="H209" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I209" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A210" s="14" t="s">
-        <v>390</v>
-      </c>
-      <c r="B210" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C210" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D210" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E210" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F210" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G210" s="14" t="n">
+      <c r="A210" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="B210" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C210" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D210" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E210" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F210" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G210" s="12" t="n">
         <v>30004</v>
       </c>
-      <c r="H210" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I210" s="14" t="s">
-        <v>379</v>
+      <c r="H210" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I210" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A211" s="14" t="s">
-        <v>391</v>
-      </c>
-      <c r="B211" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C211" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D211" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E211" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F211" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G211" s="14" t="n">
+      <c r="A211" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="B211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C211" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F211" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G211" s="12" t="n">
         <v>30005</v>
       </c>
-      <c r="H211" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I211" s="14" t="s">
-        <v>379</v>
+      <c r="H211" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I211" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A212" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="B212" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C212" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D212" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E212" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F212" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G212" s="14" t="n">
+      <c r="A212" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="B212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C212" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F212" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G212" s="12" t="n">
         <v>30006</v>
       </c>
-      <c r="H212" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I212" s="14" t="s">
-        <v>379</v>
+      <c r="H212" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I212" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A213" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="B213" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C213" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D213" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E213" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F213" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G213" s="14" t="n">
+      <c r="A213" s="12" t="s">
+        <v>399</v>
+      </c>
+      <c r="B213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C213" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F213" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G213" s="12" t="n">
         <v>40001</v>
       </c>
-      <c r="H213" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I213" s="14" t="s">
-        <v>379</v>
+      <c r="H213" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I213" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A214" s="14" t="s">
-        <v>394</v>
-      </c>
-      <c r="B214" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C214" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D214" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E214" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F214" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G214" s="14" t="n">
+      <c r="A214" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="B214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C214" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F214" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G214" s="12" t="n">
         <v>60001</v>
       </c>
-      <c r="H214" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I214" s="14" t="s">
-        <v>379</v>
+      <c r="H214" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I214" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A215" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="B215" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C215" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D215" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E215" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F215" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G215" s="14" t="n">
+      <c r="A215" s="12" t="s">
+        <v>401</v>
+      </c>
+      <c r="B215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C215" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F215" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G215" s="12" t="n">
         <v>60002</v>
       </c>
-      <c r="H215" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" s="14" t="s">
-        <v>379</v>
+      <c r="H215" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I215" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A216" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="B216" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C216" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D216" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E216" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F216" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G216" s="14" t="n">
+      <c r="A216" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="B216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C216" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F216" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G216" s="12" t="n">
         <v>60003</v>
       </c>
-      <c r="H216" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I216" s="14" t="s">
-        <v>379</v>
+      <c r="H216" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A217" s="14" t="s">
-        <v>397</v>
-      </c>
-      <c r="B217" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C217" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D217" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E217" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F217" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G217" s="14" t="n">
+      <c r="A217" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="B217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C217" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F217" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G217" s="12" t="n">
         <v>60004</v>
       </c>
-      <c r="H217" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I217" s="14" t="s">
-        <v>379</v>
+      <c r="H217" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I217" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A218" s="14" t="s">
-        <v>398</v>
-      </c>
-      <c r="B218" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C218" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D218" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E218" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F218" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G218" s="14" t="n">
+      <c r="A218" s="12" t="s">
+        <v>404</v>
+      </c>
+      <c r="B218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C218" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F218" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G218" s="12" t="n">
         <v>60005</v>
       </c>
-      <c r="H218" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I218" s="14" t="s">
-        <v>379</v>
+      <c r="H218" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A219" s="14" t="s">
-        <v>399</v>
-      </c>
-      <c r="B219" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C219" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D219" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E219" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F219" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G219" s="14" t="n">
+      <c r="A219" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="B219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C219" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F219" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G219" s="12" t="n">
         <v>60006</v>
       </c>
-      <c r="H219" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I219" s="14" t="s">
-        <v>379</v>
+      <c r="H219" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A220" s="14" t="s">
-        <v>400</v>
-      </c>
-      <c r="B220" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C220" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D220" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E220" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F220" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G220" s="14" t="n">
+      <c r="A220" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="B220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C220" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F220" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G220" s="12" t="n">
         <v>60007</v>
       </c>
-      <c r="H220" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I220" s="14" t="s">
-        <v>379</v>
+      <c r="H220" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I220" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A221" s="14" t="s">
-        <v>401</v>
-      </c>
-      <c r="B221" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C221" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D221" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E221" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F221" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G221" s="14" t="n">
+      <c r="A221" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C221" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F221" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G221" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H221" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I221" s="14" t="s">
-        <v>379</v>
+      <c r="H221" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I221" s="12" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14128,7 +14123,7 @@
     </row>
     <row r="224" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="5" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B224" s="5"/>
       <c r="C224" s="5"/>
@@ -14140,467 +14135,467 @@
       <c r="I224" s="5"/>
     </row>
     <row r="225" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A225" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="B225" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C225" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D225" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E225" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F225" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G225" s="14" t="n">
+      <c r="A225" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C225" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F225" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G225" s="12" t="n">
         <v>30001</v>
       </c>
-      <c r="H225" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I225" s="14" t="s">
+      <c r="H225" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I225" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A226" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="B226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C226" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F226" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G226" s="12" t="n">
+        <v>30002</v>
+      </c>
+      <c r="H226" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I226" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A227" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="B227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C227" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F227" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G227" s="12" t="n">
+        <v>30003</v>
+      </c>
+      <c r="H227" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I227" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A228" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="B228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C228" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F228" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G228" s="12" t="n">
+        <v>30004</v>
+      </c>
+      <c r="H228" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I228" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A229" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="B229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C229" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F229" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G229" s="12" t="n">
+        <v>30005</v>
+      </c>
+      <c r="H229" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I229" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A230" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="B230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C230" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F230" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G230" s="12" t="n">
+        <v>30006</v>
+      </c>
+      <c r="H230" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A231" s="12" t="s">
+        <v>399</v>
+      </c>
+      <c r="B231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C231" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F231" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G231" s="12" t="n">
+        <v>40001</v>
+      </c>
+      <c r="H231" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I231" s="12" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A232" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="B232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C232" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F232" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G232" s="12" t="n">
+        <v>45001</v>
+      </c>
+      <c r="H232" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I232" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A233" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="B233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C233" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F233" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G233" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H233" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I233" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A234" s="12" t="s">
+        <v>401</v>
+      </c>
+      <c r="B234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C234" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F234" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G234" s="12" t="n">
+        <v>60002</v>
+      </c>
+      <c r="H234" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I234" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A235" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="B235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C235" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F235" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G235" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H235" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I235" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A236" s="12" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="226" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A226" s="14" t="s">
-        <v>388</v>
-      </c>
-      <c r="B226" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C226" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D226" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E226" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F226" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G226" s="14" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H226" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I226" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A227" s="14" t="s">
-        <v>389</v>
-      </c>
-      <c r="B227" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C227" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D227" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E227" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F227" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G227" s="14" t="n">
-        <v>30003</v>
-      </c>
-      <c r="H227" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I227" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A228" s="14" t="s">
-        <v>390</v>
-      </c>
-      <c r="B228" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C228" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D228" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E228" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F228" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G228" s="14" t="n">
-        <v>30004</v>
-      </c>
-      <c r="H228" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I228" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="229" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A229" s="14" t="s">
-        <v>391</v>
-      </c>
-      <c r="B229" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C229" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D229" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E229" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F229" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G229" s="14" t="n">
-        <v>30005</v>
-      </c>
-      <c r="H229" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I229" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="230" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A230" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="B230" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C230" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D230" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E230" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F230" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G230" s="14" t="n">
-        <v>30006</v>
-      </c>
-      <c r="H230" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I230" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A231" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="B231" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C231" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D231" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E231" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F231" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G231" s="14" t="n">
-        <v>40001</v>
-      </c>
-      <c r="H231" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I231" s="14" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A232" s="14" t="s">
+      <c r="B236" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C236" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D236" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E236" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F236" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G236" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H236" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I236" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A237" s="12" t="s">
         <v>404</v>
       </c>
-      <c r="B232" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C232" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D232" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E232" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F232" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G232" s="14" t="n">
-        <v>45001</v>
-      </c>
-      <c r="H232" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I232" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="233" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A233" s="14" t="s">
-        <v>394</v>
-      </c>
-      <c r="B233" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C233" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D233" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E233" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F233" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G233" s="14" t="n">
-        <v>60001</v>
-      </c>
-      <c r="H233" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I233" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="234" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A234" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="B234" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C234" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D234" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E234" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F234" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G234" s="14" t="n">
-        <v>60002</v>
-      </c>
-      <c r="H234" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I234" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="235" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A235" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="B235" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C235" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D235" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E235" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F235" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G235" s="14" t="n">
-        <v>60003</v>
-      </c>
-      <c r="H235" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I235" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="236" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A236" s="14" t="s">
-        <v>397</v>
-      </c>
-      <c r="B236" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C236" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D236" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E236" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F236" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G236" s="14" t="n">
-        <v>60004</v>
-      </c>
-      <c r="H236" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I236" s="14" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="237" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A237" s="14" t="s">
-        <v>398</v>
-      </c>
-      <c r="B237" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C237" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D237" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E237" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F237" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G237" s="14" t="n">
+      <c r="B237" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C237" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D237" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E237" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F237" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G237" s="12" t="n">
         <v>60005</v>
       </c>
-      <c r="H237" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I237" s="14" t="s">
-        <v>403</v>
+      <c r="H237" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I237" s="12" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A238" s="14" t="s">
-        <v>399</v>
-      </c>
-      <c r="B238" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C238" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D238" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E238" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F238" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G238" s="14" t="n">
+      <c r="A238" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="B238" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C238" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D238" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E238" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F238" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G238" s="12" t="n">
         <v>60006</v>
       </c>
-      <c r="H238" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I238" s="14" t="s">
-        <v>403</v>
+      <c r="H238" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I238" s="12" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A239" s="14" t="s">
-        <v>400</v>
-      </c>
-      <c r="B239" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C239" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D239" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E239" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F239" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G239" s="14" t="n">
+      <c r="A239" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="B239" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C239" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D239" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E239" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F239" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G239" s="12" t="n">
         <v>60007</v>
       </c>
-      <c r="H239" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I239" s="14" t="s">
-        <v>403</v>
+      <c r="H239" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I239" s="12" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A240" s="14" t="s">
-        <v>401</v>
-      </c>
-      <c r="B240" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C240" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="D240" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E240" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F240" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="G240" s="14" t="n">
+      <c r="A240" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B240" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C240" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D240" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E240" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F240" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G240" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H240" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I240" s="14" t="s">
-        <v>403</v>
+      <c r="H240" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I240" s="12" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15294,12 +15289,12 @@
         <v>2</v>
       </c>
       <c r="I266" s="7" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A267" s="7" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B267" s="7" t="s">
         <v>75</v>
@@ -15317,18 +15312,18 @@
         <v>26</v>
       </c>
       <c r="G267" s="10" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="H267" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I267" s="7" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="28.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A268" s="7" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B268" s="7" t="s">
         <v>75</v>
@@ -15346,187 +15341,187 @@
         <v>26</v>
       </c>
       <c r="G268" s="10" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="H268" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I268" s="7" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A269" s="14" t="s">
+      <c r="A269" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="B269" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C269" s="14" t="s">
+      <c r="B269" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C269" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D269" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E269" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F269" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G269" s="14" t="s">
+      <c r="D269" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E269" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F269" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G269" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="H269" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I269" s="14" t="s">
-        <v>405</v>
+      <c r="H269" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I269" s="12" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A270" s="14" t="s">
+      <c r="A270" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B270" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C270" s="14" t="s">
+      <c r="B270" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C270" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D270" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E270" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F270" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G270" s="14" t="s">
+      <c r="D270" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E270" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F270" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G270" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="H270" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I270" s="14" t="s">
-        <v>406</v>
+      <c r="H270" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I270" s="12" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A271" s="13" t="s">
-        <v>351</v>
-      </c>
-      <c r="B271" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C271" s="14" t="s">
+      <c r="A271" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="B271" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C271" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D271" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E271" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F271" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G271" s="15" t="s">
-        <v>352</v>
-      </c>
-      <c r="H271" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I271" s="14" t="s">
-        <v>407</v>
+      <c r="D271" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E271" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F271" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G271" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="H271" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I271" s="12" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A272" s="13" t="s">
-        <v>354</v>
-      </c>
-      <c r="B272" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C272" s="14" t="s">
+      <c r="A272" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="B272" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C272" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D272" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E272" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F272" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G272" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="H272" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I272" s="14" t="s">
-        <v>408</v>
+      <c r="D272" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E272" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F272" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G272" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="H272" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I272" s="12" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A273" s="13" t="s">
-        <v>409</v>
-      </c>
-      <c r="B273" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C273" s="14" t="s">
+      <c r="A273" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="B273" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C273" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D273" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E273" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F273" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G273" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H273" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I273" s="14" t="s">
-        <v>410</v>
+      <c r="D273" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E273" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F273" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G273" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="H273" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I273" s="12" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A274" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="B274" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C274" s="14" t="s">
+      <c r="A274" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B274" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C274" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D274" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E274" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F274" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G274" s="15" t="s">
-        <v>361</v>
-      </c>
-      <c r="H274" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I274" s="14" t="s">
-        <v>362</v>
+      <c r="D274" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E274" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F274" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G274" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="H274" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I274" s="12" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -15589,43 +15584,43 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>411</v>
+      <c r="B1" s="15" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>412</v>
+      <c r="A2" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="17" t="s">
+      <c r="A3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>413</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>414</v>
+      <c r="A5" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15679,21 +15674,21 @@
       <c r="I8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>415</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
+      <c r="A9" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>195</v>
@@ -15711,18 +15706,18 @@
         <v>26</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>195</v>
@@ -15740,18 +15735,18 @@
         <v>26</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>24</v>
@@ -15769,18 +15764,18 @@
         <v>26</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>75</v>
@@ -15798,18 +15793,18 @@
         <v>26</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>75</v>
@@ -15827,18 +15822,18 @@
         <v>26</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>75</v>
@@ -15856,18 +15851,18 @@
         <v>26</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>75</v>
@@ -15885,18 +15880,18 @@
         <v>26</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>75</v>
@@ -15914,144 +15909,144 @@
         <v>26</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>433</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
+      <c r="A20" s="16" t="s">
+        <v>439</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>434</v>
-      </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
+      <c r="A21" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>435</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
+      <c r="A22" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>436</v>
-      </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
+      <c r="A23" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>437</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
+      <c r="A24" s="17" t="s">
+        <v>443</v>
+      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
-        <v>438</v>
-      </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
+      <c r="A25" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
-        <v>439</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
+      <c r="A26" s="17" t="s">
+        <v>445</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>440</v>
-      </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
+      <c r="A27" s="17" t="s">
+        <v>446</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
-        <v>441</v>
-      </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
+      <c r="A28" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>442</v>
-      </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
+      <c r="A29" s="17" t="s">
+        <v>448</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -16201,51 +16196,51 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -16266,7 +16261,7 @@
         <v>197</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>24</v>
@@ -16275,7 +16270,7 @@
         <v>110</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>100</v>
@@ -16293,13 +16288,13 @@
         <v>2</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N8" s="7"/>
     </row>
@@ -16308,7 +16303,7 @@
         <v>199</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>24</v>
@@ -16317,7 +16312,7 @@
         <v>110</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>100</v>
@@ -16335,13 +16330,13 @@
         <v>2</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N9" s="7"/>
     </row>
@@ -16350,7 +16345,7 @@
         <v>201</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>24</v>
@@ -16359,7 +16354,7 @@
         <v>110</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>200</v>
+        <v>165</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>100</v>
@@ -16377,16 +16372,16 @@
         <v>2</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>464</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="38.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16394,7 +16389,7 @@
         <v>203</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>24</v>
@@ -16403,7 +16398,7 @@
         <v>110</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>100</v>
@@ -16421,16 +16416,16 @@
         <v>2</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>466</v>
+        <v>342</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16438,7 +16433,7 @@
         <v>205</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>109</v>
@@ -16465,16 +16460,16 @@
         <v>2</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>468</v>
+        <v>343</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16482,7 +16477,7 @@
         <v>207</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>109</v>
@@ -16509,16 +16504,16 @@
         <v>2</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>470</v>
+        <v>344</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16526,7 +16521,7 @@
         <v>209</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>24</v>
@@ -16553,13 +16548,13 @@
         <v>2</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N14" s="7"/>
     </row>
@@ -16568,7 +16563,7 @@
         <v>211</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>24</v>
@@ -16577,7 +16572,7 @@
         <v>110</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>100</v>
@@ -16595,13 +16590,13 @@
         <v>2</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N15" s="7"/>
     </row>
@@ -16610,7 +16605,7 @@
         <v>213</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>24</v>
@@ -16619,7 +16614,7 @@
         <v>110</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>100</v>
@@ -16637,16 +16632,16 @@
         <v>2</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>474</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="33.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16654,7 +16649,7 @@
         <v>215</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>24</v>
@@ -16663,7 +16658,7 @@
         <v>110</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>100</v>
@@ -16681,16 +16676,16 @@
         <v>2</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>476</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16725,13 +16720,13 @@
         <v>2</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N18" s="7"/>
     </row>
@@ -16749,7 +16744,7 @@
         <v>110</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>1</v>
@@ -16767,13 +16762,13 @@
         <v>2</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N19" s="7"/>
     </row>
@@ -16827,13 +16822,13 @@
         <v>2</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N21" s="7"/>
     </row>
@@ -16869,13 +16864,13 @@
         <v>2</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N22" s="7"/>
     </row>
@@ -16911,13 +16906,13 @@
         <v>2</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N23" s="7"/>
     </row>
@@ -16953,13 +16948,13 @@
         <v>2</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N24" s="7"/>
     </row>
@@ -16995,13 +16990,13 @@
         <v>2</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N25" s="7"/>
     </row>
@@ -17037,13 +17032,13 @@
         <v>2</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N26" s="7"/>
     </row>
@@ -17079,13 +17074,13 @@
         <v>2</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N27" s="7" t="s">
         <v>236</v>
@@ -17123,13 +17118,13 @@
         <v>2</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="N28" s="7" t="s">
         <v>239</v>
@@ -17161,7 +17156,7 @@
         <v>491</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>110</v>
@@ -17185,7 +17180,7 @@
         <v>2</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L30" s="7" t="s">
         <v>492</v>
@@ -17229,7 +17224,7 @@
         <v>2</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L31" s="7" t="s">
         <v>492</v>
@@ -17273,7 +17268,7 @@
         <v>2</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L32" s="7" t="s">
         <v>492</v>
@@ -17317,7 +17312,7 @@
         <v>2</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="L33" s="7" t="s">
         <v>492</v>
@@ -17355,7 +17350,7 @@
         <v>506</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>110</v>

</xml_diff>

<commit_message>
SOCO: Improv: Add a new register in Load Not on Grid Modbus table
As per request from Jio. Also, bumped the version to v2.21.
</commit_message>
<xml_diff>
--- a/Document/CustomerFacing/SOCOModbusTable.xlsx
+++ b/Document/CustomerFacing/SOCOModbusTable.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Firmware</t>
   </si>
   <si>
-    <t xml:space="preserve">V2.19</t>
+    <t xml:space="preserve">V2.21</t>
   </si>
   <si>
     <t xml:space="preserve">Protocol</t>
@@ -2110,7 +2110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -6589,8 +6589,10 @@
       <c r="H165" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I165" s="7" t="s">
-        <v>312</v>
+      <c r="I165" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRID load-status group: exactly one of 801, 803, 819, 804, 810, 811, 812, 813 is ON at any time</t>
+        </is>
       </c>
     </row>
     <row r="166" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6623,8 +6625,10 @@
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A167" s="7" t="s">
-        <v>315</v>
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Load Not On Grid — Grid R Phase Unhealthy &amp; Y or B Phase Healthy</t>
+        </is>
       </c>
       <c r="B167" s="7" t="s">
         <v>75</v>
@@ -7063,8 +7067,10 @@
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A183" s="7" t="s">
-        <v>334</v>
+      <c r="A183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Load Not On Grid — Grid R, Y &amp; B Phase Unhealthy</t>
+        </is>
       </c>
       <c r="B183" s="7" t="s">
         <v>75</v>
@@ -7081,19 +7087,21 @@
       <c r="F183" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="G183" s="7" t="n">
-        <v>901</v>
+      <c r="G183" s="7">
+        <v>819</v>
       </c>
       <c r="H183" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I183" s="7" t="s">
-        <v>335</v>
+      <c r="I183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set when Grid R, Y and B phases are all unhealthy (total grid outage).</t>
+        </is>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>75</v>
@@ -7111,7 +7119,7 @@
         <v>252</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="H184" s="7" t="n">
         <v>1</v>
@@ -7122,7 +7130,7 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>75</v>
@@ -7140,7 +7148,7 @@
         <v>252</v>
       </c>
       <c r="G185" s="7" t="n">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="H185" s="7" t="n">
         <v>1</v>
@@ -7151,7 +7159,7 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B186" s="7" t="s">
         <v>75</v>
@@ -7169,7 +7177,7 @@
         <v>252</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="H186" s="7" t="n">
         <v>1</v>
@@ -7179,100 +7187,100 @@
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A187" s="3" t="s">
+      <c r="A187" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C187" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="D187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F187" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="G187" s="7" t="n">
+        <v>904</v>
+      </c>
+      <c r="H187" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I187" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A188" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B187" s="4" t="s">
+      <c r="B188" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C188" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D187" s="3" t="s">
+      <c r="D188" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E187" s="4" t="s">
+      <c r="E188" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F187" s="3" t="s">
+      <c r="F188" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G187" s="4" t="s">
+      <c r="G188" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H187" s="4" t="s">
+      <c r="H188" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I187" s="3" t="s">
+      <c r="I188" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A188" s="3"/>
-      <c r="B188" s="4" t="s">
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A189" s="3"/>
+      <c r="B189" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C188" s="4" t="s">
+      <c r="C189" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D188" s="3"/>
-      <c r="E188" s="4" t="s">
+      <c r="D189" s="3"/>
+      <c r="E189" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F188" s="3"/>
-      <c r="G188" s="4" t="s">
+      <c r="F189" s="3"/>
+      <c r="G189" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H188" s="4" t="s">
+      <c r="H189" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I188" s="3"/>
-    </row>
-    <row r="189" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A189" s="5" t="s">
+      <c r="I189" s="3"/>
+    </row>
+    <row r="190" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A190" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="B189" s="5"/>
-      <c r="C189" s="5"/>
-      <c r="D189" s="5"/>
-      <c r="E189" s="5"/>
-      <c r="F189" s="5"/>
-      <c r="G189" s="5"/>
-      <c r="H189" s="5"/>
-      <c r="I189" s="5"/>
-    </row>
-    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A190" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B190" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C190" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D190" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E190" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F190" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G190" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="H190" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I190" s="7" t="s">
-        <v>112</v>
-      </c>
+      <c r="B190" s="5"/>
+      <c r="C190" s="5"/>
+      <c r="D190" s="5"/>
+      <c r="E190" s="5"/>
+      <c r="F190" s="5"/>
+      <c r="G190" s="5"/>
+      <c r="H190" s="5"/>
+      <c r="I190" s="5"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="9" t="s">
-        <v>187</v>
+        <v>108</v>
       </c>
       <c r="B191" s="7" t="s">
         <v>109</v>
@@ -7290,21 +7298,21 @@
         <v>26</v>
       </c>
       <c r="G191" s="10" t="s">
-        <v>188</v>
+        <v>340</v>
       </c>
       <c r="H191" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I191" s="7" t="s">
-        <v>189</v>
+        <v>112</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="9" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="B192" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C192" s="7" t="s">
         <v>110</v>
@@ -7319,16 +7327,18 @@
         <v>26</v>
       </c>
       <c r="G192" s="10" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H192" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I192" s="7"/>
+      <c r="I192" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B193" s="7" t="s">
         <v>24</v>
@@ -7346,16 +7356,16 @@
         <v>26</v>
       </c>
       <c r="G193" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H193" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I193" s="7"/>
     </row>
-    <row r="194" customFormat="false" ht="30.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B194" s="7" t="s">
         <v>24</v>
@@ -7373,18 +7383,16 @@
         <v>26</v>
       </c>
       <c r="G194" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H194" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I194" s="7" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="195" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I194" s="7"/>
+    </row>
+    <row r="195" customFormat="false" ht="30.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B195" s="7" t="s">
         <v>24</v>
@@ -7402,21 +7410,21 @@
         <v>26</v>
       </c>
       <c r="G195" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H195" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I195" s="7" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="196" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C196" s="7" t="s">
         <v>110</v>
@@ -7431,18 +7439,18 @@
         <v>26</v>
       </c>
       <c r="G196" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H196" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I196" s="7" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="197" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B197" s="7" t="s">
         <v>109</v>
@@ -7460,21 +7468,21 @@
         <v>26</v>
       </c>
       <c r="G197" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H197" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I197" s="7" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B198" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C198" s="7" t="s">
         <v>110</v>
@@ -7489,16 +7497,18 @@
         <v>26</v>
       </c>
       <c r="G198" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H198" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I198" s="7"/>
+      <c r="I198" s="7" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B199" s="7" t="s">
         <v>24</v>
@@ -7516,16 +7526,16 @@
         <v>26</v>
       </c>
       <c r="G199" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H199" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I199" s="7"/>
     </row>
-    <row r="200" customFormat="false" ht="34.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B200" s="7" t="s">
         <v>24</v>
@@ -7543,18 +7553,16 @@
         <v>26</v>
       </c>
       <c r="G200" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H200" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I200" s="7" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="201" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I200" s="7"/>
+    </row>
+    <row r="201" customFormat="false" ht="34.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B201" s="7" t="s">
         <v>24</v>
@@ -7572,21 +7580,21 @@
         <v>26</v>
       </c>
       <c r="G201" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H201" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I201" s="7" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B202" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C202" s="7" t="s">
         <v>110</v>
@@ -7601,16 +7609,18 @@
         <v>26</v>
       </c>
       <c r="G202" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H202" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I202" s="7"/>
+      <c r="I202" s="7" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B203" s="7" t="s">
         <v>109</v>
@@ -7628,7 +7638,7 @@
         <v>26</v>
       </c>
       <c r="G203" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H203" s="7" t="n">
         <v>2</v>
@@ -7637,10 +7647,10 @@
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B204" s="7" t="s">
-        <v>222</v>
+        <v>109</v>
       </c>
       <c r="C204" s="7" t="s">
         <v>110</v>
@@ -7655,7 +7665,7 @@
         <v>26</v>
       </c>
       <c r="G204" s="10" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H204" s="7" t="n">
         <v>2</v>
@@ -7664,7 +7674,7 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B205" s="7" t="s">
         <v>222</v>
@@ -7682,7 +7692,7 @@
         <v>26</v>
       </c>
       <c r="G205" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H205" s="7" t="n">
         <v>2</v>
@@ -7691,10 +7701,10 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="9" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B206" s="7" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="C206" s="7" t="s">
         <v>110</v>
@@ -7709,7 +7719,7 @@
         <v>26</v>
       </c>
       <c r="G206" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H206" s="7" t="n">
         <v>2</v>
@@ -7718,7 +7728,7 @@
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B207" s="7" t="s">
         <v>195</v>
@@ -7736,7 +7746,7 @@
         <v>26</v>
       </c>
       <c r="G207" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H207" s="7" t="n">
         <v>2</v>
@@ -7745,10 +7755,10 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B208" s="7" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="C208" s="7" t="s">
         <v>110</v>
@@ -7763,7 +7773,7 @@
         <v>26</v>
       </c>
       <c r="G208" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H208" s="7" t="n">
         <v>2</v>
@@ -7772,7 +7782,7 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="9" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B209" s="7" t="s">
         <v>109</v>
@@ -7790,7 +7800,7 @@
         <v>26</v>
       </c>
       <c r="G209" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H209" s="7" t="n">
         <v>2</v>
@@ -7798,11 +7808,11 @@
       <c r="I209" s="7"/>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A210" s="7" t="s">
-        <v>234</v>
+      <c r="A210" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="B210" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C210" s="7" t="s">
         <v>110</v>
@@ -7817,18 +7827,16 @@
         <v>26</v>
       </c>
       <c r="G210" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H210" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I210" s="7" t="s">
-        <v>236</v>
-      </c>
+      <c r="I210" s="7"/>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B211" s="7" t="s">
         <v>75</v>
@@ -7846,18 +7854,18 @@
         <v>26</v>
       </c>
       <c r="G211" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H211" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I211" s="7" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="212" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="7" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B212" s="7" t="s">
         <v>75</v>
@@ -7875,18 +7883,18 @@
         <v>26</v>
       </c>
       <c r="G212" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H212" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I212" s="7" t="s">
-        <v>347</v>
+        <v>239</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="7" t="s">
-        <v>348</v>
+        <v>240</v>
       </c>
       <c r="B213" s="7" t="s">
         <v>75</v>
@@ -7904,18 +7912,18 @@
         <v>26</v>
       </c>
       <c r="G213" s="10" t="s">
-        <v>349</v>
+        <v>241</v>
       </c>
       <c r="H213" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I213" s="7" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="7" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B214" s="7" t="s">
         <v>75</v>
@@ -7933,12 +7941,41 @@
         <v>26</v>
       </c>
       <c r="G214" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="H214" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I214" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A215" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B215" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C215" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D215" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E215" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G215" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="H214" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I214" s="7" t="s">
+      <c r="H215" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I215" s="7" t="s">
         <v>353</v>
       </c>
     </row>
@@ -7995,11 +8032,11 @@
     <mergeCell ref="F112:F113"/>
     <mergeCell ref="I112:I113"/>
     <mergeCell ref="A114:I114"/>
-    <mergeCell ref="A187:A188"/>
-    <mergeCell ref="D187:D188"/>
-    <mergeCell ref="F187:F188"/>
-    <mergeCell ref="I187:I188"/>
-    <mergeCell ref="A189:I189"/>
+    <mergeCell ref="A188:A189"/>
+    <mergeCell ref="D188:D189"/>
+    <mergeCell ref="F188:F189"/>
+    <mergeCell ref="I188:I189"/>
+    <mergeCell ref="A190:I190"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8012,11 +8049,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I276"/>
+  <dimension ref="A1:I277"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
@@ -12752,8 +12789,10 @@
       <c r="H174" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I174" s="7" t="s">
-        <v>312</v>
+      <c r="I174" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRID load-status group: exactly one of 801, 803, 819, 804, 810, 811, 812, 813 is ON at any time</t>
+        </is>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12786,8 +12825,10 @@
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A176" s="7" t="s">
-        <v>315</v>
+      <c r="A176" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Load Not On Grid — Grid R Phase Unhealthy &amp; Y or B Phase Healthy</t>
+        </is>
       </c>
       <c r="B176" s="7" t="s">
         <v>75</v>
@@ -13226,8 +13267,10 @@
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A192" s="7" t="s">
-        <v>334</v>
+      <c r="A192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Load Not On Grid — Grid R, Y &amp; B Phase Unhealthy</t>
+        </is>
       </c>
       <c r="B192" s="7" t="s">
         <v>75</v>
@@ -13244,19 +13287,21 @@
       <c r="F192" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="G192" s="7" t="n">
-        <v>901</v>
+      <c r="G192" s="7">
+        <v>819</v>
       </c>
       <c r="H192" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I192" s="7" t="s">
-        <v>335</v>
+      <c r="I192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set when Grid R, Y and B phases are all unhealthy (total grid outage).</t>
+        </is>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B193" s="7" t="s">
         <v>75</v>
@@ -13274,7 +13319,7 @@
         <v>252</v>
       </c>
       <c r="G193" s="7" t="n">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="H193" s="7" t="n">
         <v>1</v>
@@ -13285,7 +13330,7 @@
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B194" s="7" t="s">
         <v>75</v>
@@ -13303,7 +13348,7 @@
         <v>252</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="H194" s="7" t="n">
         <v>1</v>
@@ -13314,7 +13359,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B195" s="7" t="s">
         <v>75</v>
@@ -13332,7 +13377,7 @@
         <v>252</v>
       </c>
       <c r="G195" s="7" t="n">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="H195" s="7" t="n">
         <v>1</v>
@@ -13342,100 +13387,100 @@
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A196" s="3" t="s">
+      <c r="A196" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B196" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C196" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="D196" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E196" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F196" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>904</v>
+      </c>
+      <c r="H196" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I196" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A197" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B196" s="4" t="s">
+      <c r="B197" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C196" s="4" t="s">
+      <c r="C197" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D196" s="3" t="s">
+      <c r="D197" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E196" s="4" t="s">
+      <c r="E197" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F196" s="3" t="s">
+      <c r="F197" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G196" s="4" t="s">
+      <c r="G197" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H196" s="4" t="s">
+      <c r="H197" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I196" s="3" t="s">
+      <c r="I197" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A197" s="3"/>
-      <c r="B197" s="4" t="s">
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A198" s="3"/>
+      <c r="B198" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C197" s="4" t="s">
+      <c r="C198" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D197" s="3"/>
-      <c r="E197" s="4" t="s">
+      <c r="D198" s="3"/>
+      <c r="E198" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F197" s="3"/>
-      <c r="G197" s="4" t="s">
+      <c r="F198" s="3"/>
+      <c r="G198" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H197" s="4" t="s">
+      <c r="H198" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I197" s="3"/>
-    </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A198" s="5" t="s">
+      <c r="I198" s="3"/>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A199" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="B198" s="5"/>
-      <c r="C198" s="5"/>
-      <c r="D198" s="5"/>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="5"/>
-      <c r="H198" s="5"/>
-      <c r="I198" s="5"/>
-    </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A199" s="12" t="s">
-        <v>383</v>
-      </c>
-      <c r="B199" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C199" s="12" t="s">
-        <v>251</v>
-      </c>
-      <c r="D199" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E199" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F199" s="12" t="s">
-        <v>384</v>
-      </c>
-      <c r="G199" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H199" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I199" s="12" t="s">
-        <v>385</v>
-      </c>
+      <c r="B199" s="5"/>
+      <c r="C199" s="5"/>
+      <c r="D199" s="5"/>
+      <c r="E199" s="5"/>
+      <c r="F199" s="5"/>
+      <c r="G199" s="5"/>
+      <c r="H199" s="5"/>
+      <c r="I199" s="5"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -13453,7 +13498,7 @@
         <v>384</v>
       </c>
       <c r="G200" s="12" t="n">
-        <v>20002</v>
+        <v>20001</v>
       </c>
       <c r="H200" s="12" t="n">
         <v>1</v>
@@ -13464,7 +13509,7 @@
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -13482,7 +13527,7 @@
         <v>384</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>20003</v>
+        <v>20002</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
@@ -13493,7 +13538,7 @@
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -13511,7 +13556,7 @@
         <v>384</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>20004</v>
+        <v>20003</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
@@ -13522,7 +13567,7 @@
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -13540,7 +13585,7 @@
         <v>384</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>20005</v>
+        <v>20004</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
@@ -13551,7 +13596,7 @@
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -13569,7 +13614,7 @@
         <v>384</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>20006</v>
+        <v>20005</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
@@ -13580,7 +13625,7 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -13598,7 +13643,7 @@
         <v>384</v>
       </c>
       <c r="G205" s="12" t="n">
-        <v>20007</v>
+        <v>20006</v>
       </c>
       <c r="H205" s="12" t="n">
         <v>1</v>
@@ -13609,7 +13654,7 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -13627,7 +13672,7 @@
         <v>384</v>
       </c>
       <c r="G206" s="12" t="n">
-        <v>20008</v>
+        <v>20007</v>
       </c>
       <c r="H206" s="12" t="n">
         <v>1</v>
@@ -13638,7 +13683,7 @@
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -13656,7 +13701,7 @@
         <v>384</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>30001</v>
+        <v>20008</v>
       </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
@@ -13667,7 +13712,7 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -13685,7 +13730,7 @@
         <v>384</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
@@ -13696,7 +13741,7 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -13714,7 +13759,7 @@
         <v>384</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
@@ -13725,7 +13770,7 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -13743,7 +13788,7 @@
         <v>384</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
@@ -13754,7 +13799,7 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -13772,7 +13817,7 @@
         <v>384</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
       <c r="H211" s="12" t="n">
         <v>1</v>
@@ -13783,7 +13828,7 @@
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="12" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B212" s="12" t="s">
         <v>75</v>
@@ -13801,7 +13846,7 @@
         <v>384</v>
       </c>
       <c r="G212" s="12" t="n">
-        <v>30006</v>
+        <v>30005</v>
       </c>
       <c r="H212" s="12" t="n">
         <v>1</v>
@@ -13812,7 +13857,7 @@
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B213" s="12" t="s">
         <v>75</v>
@@ -13830,7 +13875,7 @@
         <v>384</v>
       </c>
       <c r="G213" s="12" t="n">
-        <v>40001</v>
+        <v>30006</v>
       </c>
       <c r="H213" s="12" t="n">
         <v>1</v>
@@ -13841,7 +13886,7 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="12" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B214" s="12" t="s">
         <v>75</v>
@@ -13859,7 +13904,7 @@
         <v>384</v>
       </c>
       <c r="G214" s="12" t="n">
-        <v>60001</v>
+        <v>40001</v>
       </c>
       <c r="H214" s="12" t="n">
         <v>1</v>
@@ -13870,7 +13915,7 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B215" s="12" t="s">
         <v>75</v>
@@ -13888,7 +13933,7 @@
         <v>384</v>
       </c>
       <c r="G215" s="12" t="n">
-        <v>60002</v>
+        <v>60001</v>
       </c>
       <c r="H215" s="12" t="n">
         <v>1</v>
@@ -13899,7 +13944,7 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B216" s="12" t="s">
         <v>75</v>
@@ -13917,7 +13962,7 @@
         <v>384</v>
       </c>
       <c r="G216" s="12" t="n">
-        <v>60003</v>
+        <v>60002</v>
       </c>
       <c r="H216" s="12" t="n">
         <v>1</v>
@@ -13928,7 +13973,7 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="12" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B217" s="12" t="s">
         <v>75</v>
@@ -13946,7 +13991,7 @@
         <v>384</v>
       </c>
       <c r="G217" s="12" t="n">
-        <v>60004</v>
+        <v>60003</v>
       </c>
       <c r="H217" s="12" t="n">
         <v>1</v>
@@ -13957,7 +14002,7 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B218" s="12" t="s">
         <v>75</v>
@@ -13975,7 +14020,7 @@
         <v>384</v>
       </c>
       <c r="G218" s="12" t="n">
-        <v>60005</v>
+        <v>60004</v>
       </c>
       <c r="H218" s="12" t="n">
         <v>1</v>
@@ -13986,7 +14031,7 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B219" s="12" t="s">
         <v>75</v>
@@ -14004,7 +14049,7 @@
         <v>384</v>
       </c>
       <c r="G219" s="12" t="n">
-        <v>60006</v>
+        <v>60005</v>
       </c>
       <c r="H219" s="12" t="n">
         <v>1</v>
@@ -14015,7 +14060,7 @@
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B220" s="12" t="s">
         <v>75</v>
@@ -14033,7 +14078,7 @@
         <v>384</v>
       </c>
       <c r="G220" s="12" t="n">
-        <v>60007</v>
+        <v>60006</v>
       </c>
       <c r="H220" s="12" t="n">
         <v>1</v>
@@ -14044,7 +14089,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="12" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B221" s="12" t="s">
         <v>75</v>
@@ -14062,7 +14107,7 @@
         <v>384</v>
       </c>
       <c r="G221" s="12" t="n">
-        <v>60008</v>
+        <v>60007</v>
       </c>
       <c r="H221" s="12" t="n">
         <v>1</v>
@@ -14071,101 +14116,101 @@
         <v>385</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A222" s="3" t="s">
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A222" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C222" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F222" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G222" s="12" t="n">
+        <v>60008</v>
+      </c>
+      <c r="H222" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I222" s="12" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A223" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B222" s="4" t="s">
+      <c r="B223" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C222" s="4" t="s">
+      <c r="C223" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D222" s="3" t="s">
+      <c r="D223" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E222" s="4" t="s">
+      <c r="E223" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F222" s="3" t="s">
+      <c r="F223" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G222" s="4" t="s">
+      <c r="G223" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H222" s="4" t="s">
+      <c r="H223" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I222" s="3" t="s">
+      <c r="I223" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A223" s="3"/>
-      <c r="B223" s="4" t="s">
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A224" s="3"/>
+      <c r="B224" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C223" s="4" t="s">
+      <c r="C224" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D223" s="3"/>
-      <c r="E223" s="4" t="s">
+      <c r="D224" s="3"/>
+      <c r="E224" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F223" s="3"/>
-      <c r="G223" s="4" t="s">
+      <c r="F224" s="3"/>
+      <c r="G224" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H223" s="4" t="s">
+      <c r="H224" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I223" s="3"/>
-    </row>
-    <row r="224" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A224" s="5" t="s">
+      <c r="I224" s="3"/>
+    </row>
+    <row r="225" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A225" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="B224" s="5"/>
-      <c r="C224" s="5"/>
-      <c r="D224" s="5"/>
-      <c r="E224" s="5"/>
-      <c r="F224" s="5"/>
-      <c r="G224" s="5"/>
-      <c r="H224" s="5"/>
-      <c r="I224" s="5"/>
-    </row>
-    <row r="225" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A225" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="B225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C225" s="12" t="s">
-        <v>251</v>
-      </c>
-      <c r="D225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F225" s="12" t="s">
-        <v>384</v>
-      </c>
-      <c r="G225" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H225" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I225" s="12" t="s">
-        <v>409</v>
-      </c>
+      <c r="B225" s="5"/>
+      <c r="C225" s="5"/>
+      <c r="D225" s="5"/>
+      <c r="E225" s="5"/>
+      <c r="F225" s="5"/>
+      <c r="G225" s="5"/>
+      <c r="H225" s="5"/>
+      <c r="I225" s="5"/>
     </row>
     <row r="226" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="12" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B226" s="12" t="s">
         <v>75</v>
@@ -14183,7 +14228,7 @@
         <v>384</v>
       </c>
       <c r="G226" s="12" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
       <c r="H226" s="12" t="n">
         <v>1</v>
@@ -14194,7 +14239,7 @@
     </row>
     <row r="227" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="12" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B227" s="12" t="s">
         <v>75</v>
@@ -14212,7 +14257,7 @@
         <v>384</v>
       </c>
       <c r="G227" s="12" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
       <c r="H227" s="12" t="n">
         <v>1</v>
@@ -14223,7 +14268,7 @@
     </row>
     <row r="228" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="12" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B228" s="12" t="s">
         <v>75</v>
@@ -14241,7 +14286,7 @@
         <v>384</v>
       </c>
       <c r="G228" s="12" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
       <c r="H228" s="12" t="n">
         <v>1</v>
@@ -14252,7 +14297,7 @@
     </row>
     <row r="229" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B229" s="12" t="s">
         <v>75</v>
@@ -14270,7 +14315,7 @@
         <v>384</v>
       </c>
       <c r="G229" s="12" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
       <c r="H229" s="12" t="n">
         <v>1</v>
@@ -14281,7 +14326,7 @@
     </row>
     <row r="230" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="12" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B230" s="12" t="s">
         <v>75</v>
@@ -14299,7 +14344,7 @@
         <v>384</v>
       </c>
       <c r="G230" s="12" t="n">
-        <v>30006</v>
+        <v>30005</v>
       </c>
       <c r="H230" s="12" t="n">
         <v>1</v>
@@ -14308,9 +14353,9 @@
         <v>409</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B231" s="12" t="s">
         <v>75</v>
@@ -14328,18 +14373,18 @@
         <v>384</v>
       </c>
       <c r="G231" s="12" t="n">
-        <v>40001</v>
+        <v>30006</v>
       </c>
       <c r="H231" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I231" s="12" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="12" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="B232" s="12" t="s">
         <v>75</v>
@@ -14357,18 +14402,18 @@
         <v>384</v>
       </c>
       <c r="G232" s="12" t="n">
-        <v>45001</v>
+        <v>40001</v>
       </c>
       <c r="H232" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I232" s="12" t="s">
-        <v>409</v>
+        <v>385</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="12" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="B233" s="12" t="s">
         <v>75</v>
@@ -14386,7 +14431,7 @@
         <v>384</v>
       </c>
       <c r="G233" s="12" t="n">
-        <v>60001</v>
+        <v>45001</v>
       </c>
       <c r="H233" s="12" t="n">
         <v>1</v>
@@ -14397,7 +14442,7 @@
     </row>
     <row r="234" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B234" s="12" t="s">
         <v>75</v>
@@ -14415,7 +14460,7 @@
         <v>384</v>
       </c>
       <c r="G234" s="12" t="n">
-        <v>60002</v>
+        <v>60001</v>
       </c>
       <c r="H234" s="12" t="n">
         <v>1</v>
@@ -14426,7 +14471,7 @@
     </row>
     <row r="235" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B235" s="12" t="s">
         <v>75</v>
@@ -14444,7 +14489,7 @@
         <v>384</v>
       </c>
       <c r="G235" s="12" t="n">
-        <v>60003</v>
+        <v>60002</v>
       </c>
       <c r="H235" s="12" t="n">
         <v>1</v>
@@ -14455,7 +14500,7 @@
     </row>
     <row r="236" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="12" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B236" s="12" t="s">
         <v>75</v>
@@ -14473,7 +14518,7 @@
         <v>384</v>
       </c>
       <c r="G236" s="12" t="n">
-        <v>60004</v>
+        <v>60003</v>
       </c>
       <c r="H236" s="12" t="n">
         <v>1</v>
@@ -14484,7 +14529,7 @@
     </row>
     <row r="237" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B237" s="12" t="s">
         <v>75</v>
@@ -14502,7 +14547,7 @@
         <v>384</v>
       </c>
       <c r="G237" s="12" t="n">
-        <v>60005</v>
+        <v>60004</v>
       </c>
       <c r="H237" s="12" t="n">
         <v>1</v>
@@ -14513,7 +14558,7 @@
     </row>
     <row r="238" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B238" s="12" t="s">
         <v>75</v>
@@ -14531,7 +14576,7 @@
         <v>384</v>
       </c>
       <c r="G238" s="12" t="n">
-        <v>60006</v>
+        <v>60005</v>
       </c>
       <c r="H238" s="12" t="n">
         <v>1</v>
@@ -14542,7 +14587,7 @@
     </row>
     <row r="239" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B239" s="12" t="s">
         <v>75</v>
@@ -14560,7 +14605,7 @@
         <v>384</v>
       </c>
       <c r="G239" s="12" t="n">
-        <v>60007</v>
+        <v>60006</v>
       </c>
       <c r="H239" s="12" t="n">
         <v>1</v>
@@ -14571,7 +14616,7 @@
     </row>
     <row r="240" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="12" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B240" s="12" t="s">
         <v>75</v>
@@ -14589,7 +14634,7 @@
         <v>384</v>
       </c>
       <c r="G240" s="12" t="n">
-        <v>60008</v>
+        <v>60007</v>
       </c>
       <c r="H240" s="12" t="n">
         <v>1</v>
@@ -14598,101 +14643,101 @@
         <v>409</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A241" s="3" t="s">
+    <row r="241" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A241" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B241" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C241" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D241" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E241" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F241" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G241" s="12" t="n">
+        <v>60008</v>
+      </c>
+      <c r="H241" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I241" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A242" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B241" s="4" t="s">
+      <c r="B242" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C241" s="4" t="s">
+      <c r="C242" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D241" s="3" t="s">
+      <c r="D242" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E241" s="4" t="s">
+      <c r="E242" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F241" s="3" t="s">
+      <c r="F242" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G241" s="4" t="s">
+      <c r="G242" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H241" s="4" t="s">
+      <c r="H242" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I241" s="3" t="s">
+      <c r="I242" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A242" s="3"/>
-      <c r="B242" s="4" t="s">
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A243" s="3"/>
+      <c r="B243" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C242" s="4" t="s">
+      <c r="C243" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D242" s="3"/>
-      <c r="E242" s="4" t="s">
+      <c r="D243" s="3"/>
+      <c r="E243" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F242" s="3"/>
-      <c r="G242" s="4" t="s">
+      <c r="F243" s="3"/>
+      <c r="G243" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H242" s="4" t="s">
+      <c r="H243" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I242" s="3"/>
-    </row>
-    <row r="243" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A243" s="5" t="s">
+      <c r="I243" s="3"/>
+    </row>
+    <row r="244" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A244" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="B243" s="5"/>
-      <c r="C243" s="5"/>
-      <c r="D243" s="5"/>
-      <c r="E243" s="5"/>
-      <c r="F243" s="5"/>
-      <c r="G243" s="5"/>
-      <c r="H243" s="5"/>
-      <c r="I243" s="5"/>
-    </row>
-    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A244" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B244" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C244" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D244" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E244" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F244" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G244" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="H244" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I244" s="7" t="s">
-        <v>112</v>
-      </c>
+      <c r="B244" s="5"/>
+      <c r="C244" s="5"/>
+      <c r="D244" s="5"/>
+      <c r="E244" s="5"/>
+      <c r="F244" s="5"/>
+      <c r="G244" s="5"/>
+      <c r="H244" s="5"/>
+      <c r="I244" s="5"/>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="9" t="s">
-        <v>187</v>
+        <v>108</v>
       </c>
       <c r="B245" s="7" t="s">
         <v>109</v>
@@ -14710,21 +14755,21 @@
         <v>26</v>
       </c>
       <c r="G245" s="10" t="s">
-        <v>188</v>
+        <v>340</v>
       </c>
       <c r="H245" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I245" s="7" t="s">
-        <v>189</v>
+        <v>112</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="9" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C246" s="7" t="s">
         <v>110</v>
@@ -14739,16 +14784,18 @@
         <v>26</v>
       </c>
       <c r="G246" s="10" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H246" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I246" s="7"/>
+      <c r="I246" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A247" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B247" s="7" t="s">
         <v>24</v>
@@ -14766,7 +14813,7 @@
         <v>26</v>
       </c>
       <c r="G247" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H247" s="7" t="n">
         <v>2</v>
@@ -14775,7 +14822,7 @@
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A248" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B248" s="7" t="s">
         <v>24</v>
@@ -14793,7 +14840,7 @@
         <v>26</v>
       </c>
       <c r="G248" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H248" s="7" t="n">
         <v>2</v>
@@ -14802,7 +14849,7 @@
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A249" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B249" s="7" t="s">
         <v>24</v>
@@ -14820,7 +14867,7 @@
         <v>26</v>
       </c>
       <c r="G249" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H249" s="7" t="n">
         <v>2</v>
@@ -14829,10 +14876,10 @@
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A250" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B250" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C250" s="7" t="s">
         <v>110</v>
@@ -14847,7 +14894,7 @@
         <v>26</v>
       </c>
       <c r="G250" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H250" s="7" t="n">
         <v>2</v>
@@ -14856,7 +14903,7 @@
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A251" s="9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B251" s="7" t="s">
         <v>109</v>
@@ -14874,7 +14921,7 @@
         <v>26</v>
       </c>
       <c r="G251" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H251" s="7" t="n">
         <v>2</v>
@@ -14883,10 +14930,10 @@
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A252" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B252" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C252" s="7" t="s">
         <v>110</v>
@@ -14901,7 +14948,7 @@
         <v>26</v>
       </c>
       <c r="G252" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H252" s="7" t="n">
         <v>2</v>
@@ -14910,7 +14957,7 @@
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A253" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B253" s="7" t="s">
         <v>24</v>
@@ -14928,7 +14975,7 @@
         <v>26</v>
       </c>
       <c r="G253" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H253" s="7" t="n">
         <v>2</v>
@@ -14937,7 +14984,7 @@
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B254" s="7" t="s">
         <v>24</v>
@@ -14955,7 +15002,7 @@
         <v>26</v>
       </c>
       <c r="G254" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H254" s="7" t="n">
         <v>2</v>
@@ -14964,7 +15011,7 @@
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B255" s="7" t="s">
         <v>24</v>
@@ -14982,7 +15029,7 @@
         <v>26</v>
       </c>
       <c r="G255" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H255" s="7" t="n">
         <v>2</v>
@@ -14991,10 +15038,10 @@
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A256" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B256" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C256" s="7" t="s">
         <v>110</v>
@@ -15009,7 +15056,7 @@
         <v>26</v>
       </c>
       <c r="G256" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H256" s="7" t="n">
         <v>2</v>
@@ -15018,7 +15065,7 @@
     </row>
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A257" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B257" s="7" t="s">
         <v>109</v>
@@ -15036,7 +15083,7 @@
         <v>26</v>
       </c>
       <c r="G257" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H257" s="7" t="n">
         <v>2</v>
@@ -15045,10 +15092,10 @@
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A258" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B258" s="7" t="s">
-        <v>222</v>
+        <v>109</v>
       </c>
       <c r="C258" s="7" t="s">
         <v>110</v>
@@ -15063,7 +15110,7 @@
         <v>26</v>
       </c>
       <c r="G258" s="10" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H258" s="7" t="n">
         <v>2</v>
@@ -15072,7 +15119,7 @@
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A259" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B259" s="7" t="s">
         <v>222</v>
@@ -15090,7 +15137,7 @@
         <v>26</v>
       </c>
       <c r="G259" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H259" s="7" t="n">
         <v>2</v>
@@ -15099,10 +15146,10 @@
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A260" s="9" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B260" s="7" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="C260" s="7" t="s">
         <v>110</v>
@@ -15117,7 +15164,7 @@
         <v>26</v>
       </c>
       <c r="G260" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H260" s="7" t="n">
         <v>2</v>
@@ -15126,7 +15173,7 @@
     </row>
     <row r="261" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A261" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B261" s="7" t="s">
         <v>195</v>
@@ -15144,7 +15191,7 @@
         <v>26</v>
       </c>
       <c r="G261" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H261" s="7" t="n">
         <v>2</v>
@@ -15153,10 +15200,10 @@
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A262" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B262" s="7" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="C262" s="7" t="s">
         <v>110</v>
@@ -15171,7 +15218,7 @@
         <v>26</v>
       </c>
       <c r="G262" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H262" s="7" t="n">
         <v>2</v>
@@ -15180,7 +15227,7 @@
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A263" s="9" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B263" s="7" t="s">
         <v>109</v>
@@ -15198,7 +15245,7 @@
         <v>26</v>
       </c>
       <c r="G263" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H263" s="7" t="n">
         <v>2</v>
@@ -15206,11 +15253,11 @@
       <c r="I263" s="7"/>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A264" s="7" t="s">
-        <v>234</v>
+      <c r="A264" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="B264" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C264" s="7" t="s">
         <v>110</v>
@@ -15225,18 +15272,16 @@
         <v>26</v>
       </c>
       <c r="G264" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H264" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I264" s="7" t="s">
-        <v>236</v>
-      </c>
+      <c r="I264" s="7"/>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A265" s="7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B265" s="7" t="s">
         <v>75</v>
@@ -15254,18 +15299,18 @@
         <v>26</v>
       </c>
       <c r="G265" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H265" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I265" s="7" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="266" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A266" s="7" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B266" s="7" t="s">
         <v>75</v>
@@ -15283,18 +15328,18 @@
         <v>26</v>
       </c>
       <c r="G266" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H266" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I266" s="7" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="267" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="267" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A267" s="7" t="s">
-        <v>348</v>
+        <v>240</v>
       </c>
       <c r="B267" s="7" t="s">
         <v>75</v>
@@ -15312,18 +15357,18 @@
         <v>26</v>
       </c>
       <c r="G267" s="10" t="s">
-        <v>349</v>
+        <v>241</v>
       </c>
       <c r="H267" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I267" s="7" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="268" customFormat="false" ht="28.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="268" customFormat="false" ht="33.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A268" s="7" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B268" s="7" t="s">
         <v>75</v>
@@ -15341,47 +15386,47 @@
         <v>26</v>
       </c>
       <c r="G268" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="H268" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I268" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="269" customFormat="false" ht="28.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A269" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B269" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C269" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D269" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E269" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F269" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G269" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="H268" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I268" s="7" t="s">
+      <c r="H269" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I269" s="7" t="s">
         <v>353</v>
-      </c>
-    </row>
-    <row r="269" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A269" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="B269" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C269" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D269" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E269" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F269" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G269" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="H269" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I269" s="12" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A270" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B270" s="12" t="s">
         <v>75</v>
@@ -15399,18 +15444,18 @@
         <v>26</v>
       </c>
       <c r="G270" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H270" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I270" s="12" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="271" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A271" s="11" t="s">
-        <v>357</v>
+        <v>411</v>
+      </c>
+    </row>
+    <row r="271" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A271" s="12" t="s">
+        <v>245</v>
       </c>
       <c r="B271" s="12" t="s">
         <v>75</v>
@@ -15427,19 +15472,19 @@
       <c r="F271" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G271" s="13" t="s">
-        <v>358</v>
+      <c r="G271" s="12" t="s">
+        <v>246</v>
       </c>
       <c r="H271" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I271" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A272" s="11" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B272" s="12" t="s">
         <v>75</v>
@@ -15457,18 +15502,18 @@
         <v>26</v>
       </c>
       <c r="G272" s="13" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="H272" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I272" s="12" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="273" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="273" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A273" s="11" t="s">
-        <v>415</v>
+        <v>360</v>
       </c>
       <c r="B273" s="12" t="s">
         <v>75</v>
@@ -15486,18 +15531,18 @@
         <v>26</v>
       </c>
       <c r="G273" s="13" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="H273" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I273" s="12" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="274" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="274" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A274" s="11" t="s">
-        <v>366</v>
+        <v>415</v>
       </c>
       <c r="B274" s="12" t="s">
         <v>75</v>
@@ -15515,17 +15560,46 @@
         <v>26</v>
       </c>
       <c r="G274" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="H274" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I274" s="12" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="275" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A275" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B275" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C275" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D275" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E275" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F275" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G275" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="H274" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I274" s="12" t="s">
+      <c r="H275" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I275" s="12" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="275" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="276" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="277" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="A6:A7"/>
@@ -15538,21 +15612,21 @@
     <mergeCell ref="F121:F122"/>
     <mergeCell ref="I121:I122"/>
     <mergeCell ref="A123:I123"/>
-    <mergeCell ref="A196:A197"/>
-    <mergeCell ref="D196:D197"/>
-    <mergeCell ref="F196:F197"/>
-    <mergeCell ref="I196:I197"/>
-    <mergeCell ref="A198:I198"/>
-    <mergeCell ref="A222:A223"/>
-    <mergeCell ref="D222:D223"/>
-    <mergeCell ref="F222:F223"/>
-    <mergeCell ref="I222:I223"/>
-    <mergeCell ref="A224:I224"/>
-    <mergeCell ref="A241:A242"/>
-    <mergeCell ref="D241:D242"/>
-    <mergeCell ref="F241:F242"/>
-    <mergeCell ref="I241:I242"/>
-    <mergeCell ref="A243:I243"/>
+    <mergeCell ref="A197:A198"/>
+    <mergeCell ref="D197:D198"/>
+    <mergeCell ref="F197:F198"/>
+    <mergeCell ref="I197:I198"/>
+    <mergeCell ref="A199:I199"/>
+    <mergeCell ref="A223:A224"/>
+    <mergeCell ref="D223:D224"/>
+    <mergeCell ref="F223:F224"/>
+    <mergeCell ref="I223:I224"/>
+    <mergeCell ref="A225:I225"/>
+    <mergeCell ref="A242:A243"/>
+    <mergeCell ref="D242:D243"/>
+    <mergeCell ref="F242:F243"/>
+    <mergeCell ref="I242:I243"/>
+    <mergeCell ref="A244:I244"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>